<commit_message>
feat: rediseño minimalista del directorio de aliados
</commit_message>
<xml_diff>
--- a/Aliados Comerciales.xlsx
+++ b/Aliados Comerciales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JAN\Documents\App Solugan Sg\Iatf Pro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A5DDA56-2554-4DB5-9673-3C2C40A28713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{118BC071-63F7-4F2A-AFA2-24F697A51AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4A823A87-7BE4-482E-A45C-CEF8400D6EF4}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Aliado Comercial</t>
   </si>
@@ -43,18 +43,12 @@
     <t>Ciudad</t>
   </si>
   <si>
-    <t>Nota</t>
-  </si>
-  <si>
     <t>Solugan Sg - Soluciones Ganaderas</t>
   </si>
   <si>
     <t>+573147084328</t>
   </si>
   <si>
-    <t>Somos una empresa de servicios y productos especializados para ganaderia</t>
-  </si>
-  <si>
     <t>Colombia</t>
   </si>
   <si>
@@ -62,9 +56,6 @@
   </si>
   <si>
     <t>La Dorada</t>
-  </si>
-  <si>
-    <t>Contamos con cobertura operativa y capacidad de despliegue a nivel nacional e internacional.</t>
   </si>
   <si>
     <t>° Diagnostico reproductivo avanzado: 
@@ -91,6 +82,11 @@
 Ecografos
 Basculas electronicas
 Bretes para bovinos y bufalinos</t>
+  </si>
+  <si>
+    <t>En Solugan SG, transformamos unidades de producción ganadera en empresas eficientes, productivas y rentables. Diseñamos e implementamos soluciones tecnológicas y biotecnológicas avanzadas que garantizan la mejora continua de la calidad y optimizan el rendimiento financiero de su inversión.
+Disponemos de un área técnica especializada con la capacidad para asesorar y acompañar de manera integral su empresa ganadera. 
+Capacidad operativa a nivel nacional e internacional</t>
   </si>
 </sst>
 </file>
@@ -165,10 +161,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="9">
     <dxf>
       <alignment horizontal="justify" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -319,8 +312,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5F31D020-B4F5-4AF6-9D11-DD884F96546D}" name="Tabla1" displayName="Tabla1" ref="A1:H2" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A1:H2" xr:uid="{5F31D020-B4F5-4AF6-9D11-DD884F96546D}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5F31D020-B4F5-4AF6-9D11-DD884F96546D}" name="Tabla1" displayName="Tabla1" ref="A1:G2" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A1:G2" xr:uid="{5F31D020-B4F5-4AF6-9D11-DD884F96546D}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -328,17 +321,15 @@
     <filterColumn colId="4" hiddenButton="1"/>
     <filterColumn colId="5" hiddenButton="1"/>
     <filterColumn colId="6" hiddenButton="1"/>
-    <filterColumn colId="7" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{6F8236B0-4E7D-46FB-B8FD-31C45A0EB64D}" name="Aliado Comercial" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{012BB861-F84E-49B0-90FB-B28150E157C3}" name="Contacto" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{5539ECA3-1BBC-498A-AE3D-CC48DEBDE17F}" name="Descripcion" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{D4C826B1-B002-44D2-AC5C-93B21A5D41E0}" name="Productos Servicios" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{FA48978B-6610-4824-BC03-55A82893F5F8}" name="Pais" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{E45EB025-A06B-4873-8938-1321F5C37895}" name="Region" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{6185D967-8BAA-4B1E-A316-7FE6DF2DB0A1}" name="Ciudad" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{9CA47F43-0C80-4167-B5D7-4D3724287BB1}" name="Nota" dataDxfId="0"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{6F8236B0-4E7D-46FB-B8FD-31C45A0EB64D}" name="Aliado Comercial" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{012BB861-F84E-49B0-90FB-B28150E157C3}" name="Contacto" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{5539ECA3-1BBC-498A-AE3D-CC48DEBDE17F}" name="Descripcion" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{D4C826B1-B002-44D2-AC5C-93B21A5D41E0}" name="Productos Servicios" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{FA48978B-6610-4824-BC03-55A82893F5F8}" name="Pais" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{E45EB025-A06B-4873-8938-1321F5C37895}" name="Region" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{6185D967-8BAA-4B1E-A316-7FE6DF2DB0A1}" name="Ciudad" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -641,20 +632,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C28C1E06-7D81-4F80-8BA2-A7BF45497EFD}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="64.5546875" customWidth="1"/>
+    <col min="1" max="1" width="38.88671875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="34.5546875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="37.77734375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="17.33203125" customWidth="1"/>
+    <col min="3" max="3" width="57.5546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="35.44140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="12.88671875" customWidth="1"/>
     <col min="6" max="6" width="15.109375" customWidth="1"/>
     <col min="7" max="7" width="13.5546875" customWidth="1"/>
-    <col min="8" max="8" width="29.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -676,34 +666,28 @@
       <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:7" ht="388.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="388.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="F2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>11</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: encode spaces in js query params to fix script error
</commit_message>
<xml_diff>
--- a/Aliados Comerciales.xlsx
+++ b/Aliados Comerciales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JAN\Documents\App Solugan Sg\Iatf Pro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{118BC071-63F7-4F2A-AFA2-24F697A51AFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF98AB09-99E9-46D9-BFF7-3172C46B04FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4A823A87-7BE4-482E-A45C-CEF8400D6EF4}"/>
   </bookViews>
@@ -58,9 +58,15 @@
     <t>La Dorada</t>
   </si>
   <si>
+    <t>En Solugan SG, transformamos unidades de producción ganadera en empresas eficientes, productivas y rentables. Diseñamos e implementamos soluciones tecnológicas y biotecnológicas avanzadas que garantizan la mejora continua de la calidad y optimizan el rendimiento financiero de su inversión.
+Disponemos de un área técnica especializada con la capacidad para asesorar y acompañar de manera integral su empresa ganadera. 
+Capacidad operativa a nivel nacional e internacional</t>
+  </si>
+  <si>
     <t>° Diagnostico reproductivo avanzado: 
 Ultrasonografia + aplicativo Evar Pro
-° Gestion Inteligente: Monitoreo con software ganadero
+° Gestion Inteligente: 
+Monitoreo con software ganadero
 Identificacion electronica
 Auditoria de ganaderias
 ° Biotecnologias reproductivas:
@@ -82,11 +88,6 @@
 Ecografos
 Basculas electronicas
 Bretes para bovinos y bufalinos</t>
-  </si>
-  <si>
-    <t>En Solugan SG, transformamos unidades de producción ganadera en empresas eficientes, productivas y rentables. Diseñamos e implementamos soluciones tecnológicas y biotecnológicas avanzadas que garantizan la mejora continua de la calidad y optimizan el rendimiento financiero de su inversión.
-Disponemos de un área técnica especializada con la capacidad para asesorar y acompañar de manera integral su empresa ganadera. 
-Capacidad operativa a nivel nacional e internacional</t>
   </si>
 </sst>
 </file>
@@ -675,10 +676,10 @@
         <v>8</v>
       </c>
       <c r="C2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>13</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>12</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>9</v>

</xml_diff>